<commit_message>
Fix strikethrough/italic on visa Excel + shrink long agency values
- The official template's fonts carry LibreOffice <b val="0"/>, <i val="0"/>,
  <strike val="0"/> off-flags that exceljs mis-reads as ON, striking every
  cell. Strip those false-flags from the template's styles.xml so exceljs
  reads the true (off) state
- Enable shrinkToFit on the agency-info cells so a long Siège social / RC
  value fits instead of being clipped
</commit_message>
<xml_diff>
--- a/templates/assets/visa-list-template.xlsx
+++ b/templates/assets/visa-list-template.xlsx
@@ -856,64 +856,41 @@
   <numFmts count="0"/>
   <fonts count="7">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="14"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="16"/>
       <color rgb="FF339966"/>
       <name val="Times New Roman"/>

</xml_diff>